<commit_message>
Flashcards: Add Flashcard — by test_dummy
</commit_message>
<xml_diff>
--- a/Subject_Scheduler.xlsx
+++ b/Subject_Scheduler.xlsx
@@ -2139,7 +2139,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H157"/>
+  <dimension ref="A1:H158"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -6181,16 +6181,42 @@
         <v>2026-09-06T10:47:29.127Z</v>
       </c>
     </row>
+    <row r="158">
+      <c r="A158" t="str">
+        <v>card_1789676513729_4y0fau</v>
+      </c>
+      <c r="B158" t="str">
+        <v>EA - IS105 - Week4 - 6 (UML Diagrams)</v>
+      </c>
+      <c r="C158" t="str">
+        <v>basic</v>
+      </c>
+      <c r="D158" t="str">
+        <v>It is a valuable tool in Unified Modeling Language (UML) for visually representing the flow of control within a system.</v>
+      </c>
+      <c r="E158" t="str">
+        <v>Activity Diagram</v>
+      </c>
+      <c r="F158" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="G158" t="str">
+        <v>2026-09-17T20:21:53.729Z</v>
+      </c>
+      <c r="H158" t="str">
+        <v>2026-09-17T20:21:53.729Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H157"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H158"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E247"/>
+  <dimension ref="A1:E250"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -10357,9 +10383,60 @@
         <v>ADV01 - Intro to EntSys n Mang. — cloze</v>
       </c>
     </row>
+    <row r="248">
+      <c r="A248" t="str">
+        <v>2026-09-18T03:45:56+08:00</v>
+      </c>
+      <c r="B248" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="C248" t="str">
+        <v>Master</v>
+      </c>
+      <c r="D248" t="str">
+        <v>Login</v>
+      </c>
+      <c r="E248" t="str">
+        <v>Master</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="str">
+        <v>2026-09-18T03:46:12+08:00</v>
+      </c>
+      <c r="B249" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="C249" t="str">
+        <v>Master</v>
+      </c>
+      <c r="D249" t="str">
+        <v>Login</v>
+      </c>
+      <c r="E249" t="str">
+        <v>Master</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="str">
+        <v>2026-09-18T04:21:53+08:00</v>
+      </c>
+      <c r="B250" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="C250" t="str">
+        <v>Master</v>
+      </c>
+      <c r="D250" t="str">
+        <v>Add Flashcard</v>
+      </c>
+      <c r="E250" t="str">
+        <v>EA - IS105 - Week4 - 6 (UML Diagrams)</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E247"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E250"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Audit: Login — by Bert
</commit_message>
<xml_diff>
--- a/Subject_Scheduler.xlsx
+++ b/Subject_Scheduler.xlsx
@@ -2111,16 +2111,6 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H524"/>
-  <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="26.83203125" customWidth="1"/>
-    <col min="3" max="3" width="10.83203125" customWidth="1"/>
-    <col min="4" max="4" width="40.83203125" customWidth="1"/>
-    <col min="5" max="5" width="40.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="20.83203125" customWidth="1"/>
-    <col min="8" max="8" width="20.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -15917,7 +15907,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E370"/>
+  <dimension ref="A1:E371"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -22175,9 +22165,26 @@
         <v>278 cards — 3rd_year / Midterm / ADV01 / Lesson 6 SDLC, 3rd_year / Midterm / ADV01 / WEEK 1, 3rd_year / Midterm / ADV01 / WEEK 2, 3rd_year / Midterm / ADV01 / WEEK 3, 3rd_year / Midterm / ADV01 / WEEK 6 - SDLC</v>
       </c>
     </row>
+    <row r="371">
+      <c r="A371" t="str">
+        <v>2026-10-11T12:30:04+08:00</v>
+      </c>
+      <c r="B371" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="C371" t="str">
+        <v>Master</v>
+      </c>
+      <c r="D371" t="str">
+        <v>Login</v>
+      </c>
+      <c r="E371" t="str">
+        <v>Master</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E370"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E371"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -22233,11 +22240,6 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C13"/>
-  <cols>
-    <col min="1" max="1" width="60.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>

<commit_message>
Flashcards: Add Flashcards (drafted) — by Bert
</commit_message>
<xml_diff>
--- a/Subject_Scheduler.xlsx
+++ b/Subject_Scheduler.xlsx
@@ -2110,7 +2110,17 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H524"/>
+  <dimension ref="A1:H537"/>
+  <cols>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="26.83203125" customWidth="1"/>
+    <col min="3" max="3" width="10.83203125" customWidth="1"/>
+    <col min="4" max="4" width="40.83203125" customWidth="1"/>
+    <col min="5" max="5" width="40.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" customWidth="1"/>
+    <col min="8" max="8" width="20.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -15898,16 +15908,367 @@
         <v>2026-10-05T12:11:35.944Z</v>
       </c>
     </row>
+    <row r="525" xml:space="preserve">
+      <c r="A525" t="str">
+        <v>card_1791696321508_bddrsl</v>
+      </c>
+      <c r="B525" t="str">
+        <v>3rd_year / Midterm / ADV01 / Week1 - Introduction to ESnM</v>
+      </c>
+      <c r="C525" t="str">
+        <v>basic</v>
+      </c>
+      <c r="D525" t="str">
+        <v>What are the three(3) Levels of Management?</v>
+      </c>
+      <c r="E525" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Administrative, Managerial, or Top Level of Management
+• Executive or Middle Level of Management
+• Supervisory, Operative, or Lower Level of Management</v>
+      </c>
+      <c r="F525" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="G525" t="str">
+        <v>2026-10-11T05:25:23.235Z</v>
+      </c>
+      <c r="H525" t="str">
+        <v>2026-10-11T05:25:23.235Z</v>
+      </c>
+    </row>
+    <row r="526" xml:space="preserve">
+      <c r="A526" t="str">
+        <v>card_1791696321508_pnm1fu</v>
+      </c>
+      <c r="B526" t="str">
+        <v>3rd_year / Midterm / ADV01 / Week1 - Introduction to ESnM</v>
+      </c>
+      <c r="C526" t="str">
+        <v>basic</v>
+      </c>
+      <c r="D526" t="str" xml:space="preserve">
+        <v xml:space="preserve">&lt;!--rt--&gt;It is the ultimate source of power and authority since it oversees a company's goals, policies, and procedures.
+&lt;span style="color:#0f766e"&gt;#-Level of Management&lt;/span&gt;</v>
+      </c>
+      <c r="E526" t="str">
+        <v>Administrative, Managerial, or Top Level of Management</v>
+      </c>
+      <c r="F526" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="G526" t="str">
+        <v>2026-10-11T05:25:23.235Z</v>
+      </c>
+      <c r="H526" t="str">
+        <v>2026-10-11T05:25:23.235Z</v>
+      </c>
+    </row>
+    <row r="527" xml:space="preserve">
+      <c r="A527" t="str">
+        <v>card_1791696321508_c6huxx</v>
+      </c>
+      <c r="B527" t="str">
+        <v>3rd_year / Midterm / ADV01 / Week1 - Introduction to ESnM</v>
+      </c>
+      <c r="C527" t="str">
+        <v>basic</v>
+      </c>
+      <c r="D527" t="str" xml:space="preserve">
+        <v xml:space="preserve">&lt;!--rt--&gt;The branch and departmental managers form this middle management level.
+&lt;span style="color:#0f766e"&gt;#-Level of Management&lt;/span&gt;</v>
+      </c>
+      <c r="E527" t="str">
+        <v>Executive or Middle Level of Management</v>
+      </c>
+      <c r="F527" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="G527" t="str">
+        <v>2026-10-11T05:25:23.235Z</v>
+      </c>
+      <c r="H527" t="str">
+        <v>2026-10-11T05:25:23.235Z</v>
+      </c>
+    </row>
+    <row r="528" xml:space="preserve">
+      <c r="A528" t="str">
+        <v>card_1791696321508_y17yn7</v>
+      </c>
+      <c r="B528" t="str">
+        <v>3rd_year / Midterm / ADV01 / Week1 - Introduction to ESnM</v>
+      </c>
+      <c r="C528" t="str">
+        <v>basic</v>
+      </c>
+      <c r="D528" t="str" xml:space="preserve">
+        <v xml:space="preserve">&lt;!--rt--&gt;This management level consists of supervisors, foremen, section officers, superintendents, and all other executives whose work must do largely with HR oversight and the direction of operative employees. &lt;b&gt;Managers&lt;/b&gt; at the lower level are primarily concerned with the execution and coordination of day-to-day workflow that ensures the completion of projects and that deliverables are met.
+&lt;span style="color:#0f766e"&gt;#-Level of Management&lt;/span&gt;</v>
+      </c>
+      <c r="E528" t="str">
+        <v>Supervisory, Operative, or Lower Level of Management</v>
+      </c>
+      <c r="F528" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="G528" t="str">
+        <v>2026-10-11T05:25:23.235Z</v>
+      </c>
+      <c r="H528" t="str">
+        <v>2026-10-11T05:25:23.235Z</v>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="str">
+        <v>card_1791696321508_r4q1qi</v>
+      </c>
+      <c r="B529" t="str">
+        <v>3rd_year / Midterm / ADV01 / Week1 - Introduction to ESnM</v>
+      </c>
+      <c r="C529" t="str">
+        <v>cloze</v>
+      </c>
+      <c r="D529" t="str">
+        <v>_____ systems are the specific kind of enterprise systems to integrate data across and be comprehensive in supporting all the organization's major functions. ERP systems are comprehensive software applications that support critical organizational functions.</v>
+      </c>
+      <c r="E529" t="str">
+        <v>Enterprise resource planning (ERP)</v>
+      </c>
+      <c r="F529" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="G529" t="str">
+        <v>2026-10-11T05:25:23.235Z</v>
+      </c>
+      <c r="H529" t="str">
+        <v>2026-10-11T05:25:23.235Z</v>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="str">
+        <v>card_1791696321508_bs6u64</v>
+      </c>
+      <c r="B530" t="str">
+        <v>3rd_year / Midterm / ADV01 / Week1 - Introduction to ESnM</v>
+      </c>
+      <c r="C530" t="str">
+        <v>basic</v>
+      </c>
+      <c r="D530" t="str">
+        <v>&lt;!--rt--&gt;These systems were designed to manage and tract &lt;i&gt;inventory&lt;/i&gt; of raw materials and guide plan supervisors on purchase orders, alerts, and targets, providing replenishment techniques and options, inventory reconciliation, and inventory reports.</v>
+      </c>
+      <c r="E530" t="str">
+        <v>Inventory Management and Control - 1960s</v>
+      </c>
+      <c r="F530" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="G530" t="str">
+        <v>2026-10-11T05:25:23.235Z</v>
+      </c>
+      <c r="H530" t="str">
+        <v>2026-10-11T05:25:23.235Z</v>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="str">
+        <v>card_1791696321508_z5g4mj</v>
+      </c>
+      <c r="B531" t="str">
+        <v>3rd_year / Midterm / ADV01 / Week1 - Introduction to ESnM</v>
+      </c>
+      <c r="C531" t="str">
+        <v>basic</v>
+      </c>
+      <c r="D531" t="str">
+        <v>&lt;!--rt--&gt;These systems were designed for &lt;b&gt;job shop scheduling&lt;/b&gt;.</v>
+      </c>
+      <c r="E531" t="str">
+        <v>Material Requirements Planning (MRP) - 1970s</v>
+      </c>
+      <c r="F531" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="G531" t="str">
+        <v>2026-10-11T05:25:23.235Z</v>
+      </c>
+      <c r="H531" t="str">
+        <v>2026-10-11T05:25:23.235Z</v>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="str">
+        <v>card_1791696321508_8jifsf</v>
+      </c>
+      <c r="B532" t="str">
+        <v>3rd_year / Midterm / ADV01 / Week1 - Introduction to ESnM</v>
+      </c>
+      <c r="C532" t="str">
+        <v>basic</v>
+      </c>
+      <c r="D532" t="str">
+        <v>&lt;!--rt--&gt;These systems were designed for helping production managers in &lt;u&gt;designing production supply chain processes&lt;/u&gt;—from product planning, parts purchasing, inventory control, and overhead cost management to product distribution.</v>
+      </c>
+      <c r="E532" t="str">
+        <v>Manufacturing Requirements Planning II (MRP) - 1980s</v>
+      </c>
+      <c r="F532" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="G532" t="str">
+        <v>2026-10-11T05:25:23.235Z</v>
+      </c>
+      <c r="H532" t="str">
+        <v>2026-10-11T05:25:23.235Z</v>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="str">
+        <v>card_1791696321508_6pkqrb</v>
+      </c>
+      <c r="B533" t="str">
+        <v>3rd_year / Midterm / ADV01 / Week1 - Introduction to ESnM</v>
+      </c>
+      <c r="C533" t="str">
+        <v>basic</v>
+      </c>
+      <c r="D533" t="str">
+        <v>&lt;!--rt--&gt;These systems were designed for improving the performance of the internal business processes across the complete value chain of the organization. They &lt;b&gt;&lt;i&gt;integrate primary business activities&lt;/i&gt;&lt;/b&gt; like product planning, purchasing, logistics control, distribution, fulfillment, and sales; additionally, they integrate secondary or support activities like marketing, finance, accounting, and human resources.</v>
+      </c>
+      <c r="E533" t="str">
+        <v>Enterprise Resource Planning (ERP) - 1990s</v>
+      </c>
+      <c r="F533" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="G533" t="str">
+        <v>2026-10-11T05:25:23.235Z</v>
+      </c>
+      <c r="H533" t="str">
+        <v>2026-10-11T05:25:23.235Z</v>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="str">
+        <v>card_1791696321508_htt5qm</v>
+      </c>
+      <c r="B534" t="str">
+        <v>3rd_year / Midterm / ADV01 / Week1 - Introduction to ESnM</v>
+      </c>
+      <c r="C534" t="str">
+        <v>basic</v>
+      </c>
+      <c r="D534" t="str">
+        <v>&lt;!--rt--&gt;These systems focus on agility and a customer-centric global environment, these systems &lt;u&gt;extended the first-generation ERP&lt;/u&gt;.</v>
+      </c>
+      <c r="E534" t="str">
+        <v>Extended ERP or ERP II - 2000s</v>
+      </c>
+      <c r="F534" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="G534" t="str">
+        <v>2026-10-11T05:25:23.235Z</v>
+      </c>
+      <c r="H534" t="str">
+        <v>2026-10-11T05:25:23.235Z</v>
+      </c>
+    </row>
+    <row r="535" xml:space="preserve">
+      <c r="A535" t="str">
+        <v>card_1791696321508_3my4f1</v>
+      </c>
+      <c r="B535" t="str">
+        <v>3rd_year / Midterm / ADV01 / Week1 - Introduction to ESnM</v>
+      </c>
+      <c r="C535" t="str">
+        <v>basic</v>
+      </c>
+      <c r="D535" t="str">
+        <v>Enumerate the Evolution of ERP</v>
+      </c>
+      <c r="E535" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Inventory Management and Control - 1960s
+• Material Requirements Planning (MRP) - 1970s
+• Manufacturing Requirements Planning (MRP II) - 1980s
+• Enterprise Resource Planning (ERP) - 1990s
+• Extended ERP or ERP II - 2000s</v>
+      </c>
+      <c r="F535" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="G535" t="str">
+        <v>2026-10-11T05:25:23.235Z</v>
+      </c>
+      <c r="H535" t="str">
+        <v>2026-10-11T05:25:23.235Z</v>
+      </c>
+    </row>
+    <row r="536" xml:space="preserve">
+      <c r="A536" t="str">
+        <v>card_1791696321508_jj97z2</v>
+      </c>
+      <c r="B536" t="str">
+        <v>3rd_year / Midterm / ADV01 / Week1 - Introduction to ESnM</v>
+      </c>
+      <c r="C536" t="str">
+        <v>basic</v>
+      </c>
+      <c r="D536" t="str">
+        <v>Enumerate the Five(5) ERP System Components</v>
+      </c>
+      <c r="E536" t="str" xml:space="preserve">
+        <v xml:space="preserve">&lt;!--rt--&gt;&lt;span style="color:#2563eb"&gt;• Hardware&lt;/span&gt;
+&lt;span style="color:#15803d"&gt;• Software&lt;/span&gt;
+&lt;span style="color:#dc2626"&gt;• Database&lt;/span&gt;
+• Processes
+&lt;span style="color:#0f766e"&gt;• People(User)&lt;/span&gt;</v>
+      </c>
+      <c r="F536" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="G536" t="str">
+        <v>2026-10-11T05:25:23.235Z</v>
+      </c>
+      <c r="H536" t="str">
+        <v>2026-10-11T05:25:23.235Z</v>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="str">
+        <v>card_1791696321508_goefr4</v>
+      </c>
+      <c r="B537" t="str">
+        <v>3rd_year / Midterm / ADV01 / Week1 - Introduction to ESnM</v>
+      </c>
+      <c r="C537" t="str">
+        <v>cloze</v>
+      </c>
+      <c r="D537" t="str">
+        <v>A _____ is a blueprint of the actual ERP system and transforms the high-level ERP implementation strategy into an information flow with interrelationships in the organization. The process of designing _____ is slightly different from other IT architectures.</v>
+      </c>
+      <c r="E537" t="str">
+        <v>system’s architecture ‖ ERP system architecture</v>
+      </c>
+      <c r="F537" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="G537" t="str">
+        <v>2026-10-11T05:25:23.235Z</v>
+      </c>
+      <c r="H537" t="str">
+        <v>2026-10-11T05:25:23.235Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H524"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H537"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E373"/>
+  <dimension ref="A1:E374"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -22216,9 +22577,26 @@
         <v>Master</v>
       </c>
     </row>
+    <row r="374">
+      <c r="A374" t="str">
+        <v>2026-10-11T13:25:25+08:00</v>
+      </c>
+      <c r="B374" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="C374" t="str">
+        <v>Master</v>
+      </c>
+      <c r="D374" t="str">
+        <v>Add Flashcards (drafted)</v>
+      </c>
+      <c r="E374" t="str">
+        <v>13 cards to 3rd_year / Midterm / ADV01 / Week1 - Introduction to ESnM</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E373"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E374"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Flashcards: Add Flashcard — by Bert
</commit_message>
<xml_diff>
--- a/Subject_Scheduler.xlsx
+++ b/Subject_Scheduler.xlsx
@@ -2110,7 +2110,17 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H586"/>
+  <dimension ref="A1:H587"/>
+  <cols>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="26.83203125" customWidth="1"/>
+    <col min="3" max="3" width="10.83203125" customWidth="1"/>
+    <col min="4" max="4" width="40.83203125" customWidth="1"/>
+    <col min="5" max="5" width="40.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" customWidth="1"/>
+    <col min="8" max="8" width="20.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -17574,16 +17584,42 @@
         <v>2026-10-11T05:27:36.548Z</v>
       </c>
     </row>
+    <row r="587">
+      <c r="A587" t="str">
+        <v>card_1791700792581_vox3gm</v>
+      </c>
+      <c r="B587" t="str">
+        <v>3rd_year / Midterm / FIL101 / Aralin1</v>
+      </c>
+      <c r="C587" t="str">
+        <v>cloze</v>
+      </c>
+      <c r="D587" t="str">
+        <v>&lt;!--rt--&gt;Ang _____ ay tumutukoy sa isang &lt;u&gt;wikang ginagamit&lt;/u&gt; nang pasalita at pasulat ng mga &lt;span style="font-weight:bold"&gt;&lt;u&gt;mamamayan ng isang bansa.&lt;/u&gt;&lt;/span&gt; Ito ang nag-iisang wikang ginagamit batay sa kultura ng lipunan.</v>
+      </c>
+      <c r="E587" t="str">
+        <v>Wikang Pambansa</v>
+      </c>
+      <c r="F587" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="G587" t="str">
+        <v>2026-10-11T06:39:52.581Z</v>
+      </c>
+      <c r="H587" t="str">
+        <v>2026-10-11T06:39:52.581Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H586"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H587"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E380"/>
+  <dimension ref="A1:E381"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -24011,9 +24047,26 @@
         <v>Master</v>
       </c>
     </row>
+    <row r="381">
+      <c r="A381" t="str">
+        <v>2026-10-11T14:39:52+08:00</v>
+      </c>
+      <c r="B381" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="C381" t="str">
+        <v>Master</v>
+      </c>
+      <c r="D381" t="str">
+        <v>Add Flashcard</v>
+      </c>
+      <c r="E381" t="str">
+        <v>3rd_year / Midterm / FIL101 / Aralin1 — cloze</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E380"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E381"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -24069,6 +24122,11 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C13"/>
+  <cols>
+    <col min="1" max="1" width="60.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>

<commit_message>
Flashcards: Remove Empty Deck — by Bert
</commit_message>
<xml_diff>
--- a/Subject_Scheduler.xlsx
+++ b/Subject_Scheduler.xlsx
@@ -2111,6 +2111,16 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H631"/>
+  <cols>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="26.83203125" customWidth="1"/>
+    <col min="3" max="3" width="10.83203125" customWidth="1"/>
+    <col min="4" max="4" width="40.83203125" customWidth="1"/>
+    <col min="5" max="5" width="40.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" customWidth="1"/>
+    <col min="8" max="8" width="20.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -18766,7 +18776,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E402"/>
+  <dimension ref="A1:E403"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -25568,9 +25578,26 @@
         <v>Master</v>
       </c>
     </row>
+    <row r="403">
+      <c r="A403" t="str">
+        <v>2026-10-11T14:47:00+08:00</v>
+      </c>
+      <c r="B403" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="C403" t="str">
+        <v>Master</v>
+      </c>
+      <c r="D403" t="str">
+        <v>Remove Empty Deck</v>
+      </c>
+      <c r="E403" t="str">
+        <v>3rd_year / Finals</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E402"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E403"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -25625,7 +25652,12 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C12"/>
+  <cols>
+    <col min="1" max="1" width="60.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -25736,20 +25768,9 @@
         <v>2026-10-03T08:54:15.036Z</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>3rd_year / Finals</v>
-      </c>
-      <c r="B13" t="str">
-        <v>Bert</v>
-      </c>
-      <c r="C13" t="str">
-        <v>2026-10-03T08:57:58.561Z</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C12"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Flashcards: Create Deck — by Bert
</commit_message>
<xml_diff>
--- a/Subject_Scheduler.xlsx
+++ b/Subject_Scheduler.xlsx
@@ -2111,6 +2111,16 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H937"/>
+  <cols>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="26.83203125" customWidth="1"/>
+    <col min="3" max="3" width="10.83203125" customWidth="1"/>
+    <col min="4" max="4" width="40.83203125" customWidth="1"/>
+    <col min="5" max="5" width="40.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" customWidth="1"/>
+    <col min="8" max="8" width="20.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -27002,7 +27012,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E411"/>
+  <dimension ref="A1:E413"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -33957,9 +33967,43 @@
         <v>Master</v>
       </c>
     </row>
+    <row r="412">
+      <c r="A412" t="str">
+        <v>2026-10-13T12:54:04+08:00</v>
+      </c>
+      <c r="B412" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="C412" t="str">
+        <v>Master</v>
+      </c>
+      <c r="D412" t="str">
+        <v>Login</v>
+      </c>
+      <c r="E412" t="str">
+        <v>Master</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="str">
+        <v>2026-10-13T12:55:49+08:00</v>
+      </c>
+      <c r="B413" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="C413" t="str">
+        <v>Master</v>
+      </c>
+      <c r="D413" t="str">
+        <v>Create Deck</v>
+      </c>
+      <c r="E413" t="str">
+        <v>3rd_Year / Finlas</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E411"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E413"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -34014,7 +34058,12 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
+  <cols>
+    <col min="1" max="1" width="60.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -34114,9 +34163,20 @@
         <v>2026-10-03T08:54:15.036Z</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>3rd_Year / Finlas</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="C12" t="str">
+        <v>2026-10-13T04:55:48.830Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C12"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Flashcards: Edit Flashcard — by Bert
</commit_message>
<xml_diff>
--- a/Subject_Scheduler.xlsx
+++ b/Subject_Scheduler.xlsx
@@ -17132,7 +17132,7 @@
         <v>basic</v>
       </c>
       <c r="D562" t="str">
-        <v>Organizations also divided roles in hierarchical layers from strategic planning to management control and operation control.</v>
+        <v>&lt;!--rt--&gt;Organizations also divided roles in hierarchical layers from &lt;span style="color:#dc2626;background-color:#fde047;font-weight:bold"&gt;strategic planning &lt;/span&gt;to &lt;span style="font-weight:bold"&gt;&lt;span style="color:#dc2626;background-color:#86efac"&gt;management control &lt;/span&gt;and &lt;span style="color:#dc2626;background-color:#93c5fd"&gt;operation control&lt;/span&gt;&lt;/span&gt;.</v>
       </c>
       <c r="E562" t="str">
         <v>Vertical Silos</v>
@@ -17144,7 +17144,7 @@
         <v>2026-10-11T05:26:30.400Z</v>
       </c>
       <c r="H562" t="str">
-        <v>2026-10-11T05:26:30.400Z</v>
+        <v>2026-10-19T15:14:50.160Z</v>
       </c>
     </row>
     <row r="563" xml:space="preserve">
@@ -32328,7 +32328,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E34"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -32857,9 +32857,26 @@
         <v>3rd_year / Midterm / ADV01 / Week4 - 5 - ESA — Overview of Modules</v>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>2026-10-19T23:14:50+08:00</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Bert</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Master</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Edit Flashcard</v>
+      </c>
+      <c r="E34" t="str">
+        <v>3rd_year / Midterm / ADV01 / Week3 - System Integration</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E33"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E34"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>